<commit_message>
fix SS9 display error
</commit_message>
<xml_diff>
--- a/PCB/BOM-Chart.xlsx
+++ b/PCB/BOM-Chart.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xinghening/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xinghening/rp2040-lbj-project/PCB/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9E2FBC8A-B58A-4A49-88E2-4E5888C0A076}" xr6:coauthVersionLast="40" xr6:coauthVersionMax="40" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3588D1B2-9EE4-1F4E-8B34-6CD7563A48F9}" xr6:coauthVersionLast="40" xr6:coauthVersionMax="40" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1100" yWindow="820" windowWidth="28040" windowHeight="17440" xr2:uid="{EA1724DA-C935-284F-B749-F4406051A4F4}"/>
+    <workbookView xWindow="680" yWindow="1120" windowWidth="28040" windowHeight="17440" xr2:uid="{EA1724DA-C935-284F-B749-F4406051A4F4}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="78">
   <si>
     <t>位号</t>
   </si>
@@ -104,9 +104,6 @@
     <t>C0603</t>
   </si>
   <si>
-    <t>C4</t>
-  </si>
-  <si>
     <t>0.1uf</t>
   </si>
   <si>
@@ -206,9 +203,6 @@
     <t>0905</t>
   </si>
   <si>
-    <t>U6</t>
-  </si>
-  <si>
     <t>SOD323</t>
   </si>
   <si>
@@ -261,6 +255,15 @@
   </si>
   <si>
     <t>1个，屏幕的SD卡引脚通常不焊排针，需要自己焊上</t>
+  </si>
+  <si>
+    <t>C3,C4</t>
+  </si>
+  <si>
+    <t>U0</t>
+  </si>
+  <si>
+    <t>U6,U9,U10</t>
   </si>
 </sst>
 </file>
@@ -642,8 +645,8 @@
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A2">
-        <v>1</v>
+      <c r="A2" t="s">
+        <v>76</v>
       </c>
       <c r="B2" t="s">
         <v>4</v>
@@ -737,10 +740,10 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
+        <v>75</v>
+      </c>
+      <c r="B10" t="s">
         <v>24</v>
-      </c>
-      <c r="B10" t="s">
-        <v>25</v>
       </c>
       <c r="C10" t="s">
         <v>23</v>
@@ -748,166 +751,166 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
+        <v>25</v>
+      </c>
+      <c r="B11" t="s">
         <v>26</v>
       </c>
-      <c r="B11" t="s">
+      <c r="C11" t="s">
         <v>27</v>
-      </c>
-      <c r="C11" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
+        <v>28</v>
+      </c>
+      <c r="B12" t="s">
         <v>29</v>
       </c>
-      <c r="B12" t="s">
+      <c r="C12" t="s">
         <v>30</v>
-      </c>
-      <c r="C12" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
+        <v>31</v>
+      </c>
+      <c r="B13" t="s">
+        <v>4</v>
+      </c>
+      <c r="C13" t="s">
         <v>32</v>
       </c>
-      <c r="B13" t="s">
-        <v>4</v>
-      </c>
-      <c r="C13" t="s">
+      <c r="D13" t="s">
         <v>33</v>
-      </c>
-      <c r="D13" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
+        <v>34</v>
+      </c>
+      <c r="B14" t="s">
+        <v>4</v>
+      </c>
+      <c r="C14" t="s">
+        <v>32</v>
+      </c>
+      <c r="D14" t="s">
         <v>35</v>
-      </c>
-      <c r="B14" t="s">
-        <v>4</v>
-      </c>
-      <c r="C14" t="s">
-        <v>33</v>
-      </c>
-      <c r="D14" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
+        <v>36</v>
+      </c>
+      <c r="B15" t="s">
+        <v>4</v>
+      </c>
+      <c r="C15" t="s">
         <v>37</v>
       </c>
-      <c r="B15" t="s">
-        <v>4</v>
-      </c>
-      <c r="C15" t="s">
-        <v>38</v>
-      </c>
       <c r="D15" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
+        <v>38</v>
+      </c>
+      <c r="B16" t="s">
         <v>39</v>
       </c>
-      <c r="B16" t="s">
+      <c r="C16" t="s">
         <v>40</v>
       </c>
-      <c r="C16" t="s">
+      <c r="D16" t="s">
         <v>41</v>
-      </c>
-      <c r="D16" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
+        <v>42</v>
+      </c>
+      <c r="B17" t="s">
         <v>43</v>
       </c>
-      <c r="B17" t="s">
+      <c r="C17" t="s">
+        <v>40</v>
+      </c>
+      <c r="D17" t="s">
         <v>44</v>
-      </c>
-      <c r="C17" t="s">
-        <v>41</v>
-      </c>
-      <c r="D17" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
+        <v>45</v>
+      </c>
+      <c r="B18" t="s">
+        <v>4</v>
+      </c>
+      <c r="C18" t="s">
         <v>46</v>
       </c>
-      <c r="B18" t="s">
-        <v>4</v>
-      </c>
-      <c r="C18" t="s">
+      <c r="D18" t="s">
         <v>47</v>
-      </c>
-      <c r="D18" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
+        <v>48</v>
+      </c>
+      <c r="B19" t="s">
+        <v>4</v>
+      </c>
+      <c r="C19" t="s">
         <v>49</v>
       </c>
-      <c r="B19" t="s">
-        <v>4</v>
-      </c>
-      <c r="C19" t="s">
+      <c r="D19" t="s">
         <v>50</v>
-      </c>
-      <c r="D19" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
+        <v>51</v>
+      </c>
+      <c r="B20" t="s">
         <v>52</v>
       </c>
-      <c r="B20" t="s">
-        <v>53</v>
-      </c>
       <c r="C20" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
+        <v>53</v>
+      </c>
+      <c r="B21" t="s">
         <v>54</v>
       </c>
-      <c r="B21" t="s">
+      <c r="C21" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="D21" t="s">
         <v>55</v>
-      </c>
-      <c r="C21" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="D21" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
+        <v>77</v>
+      </c>
+      <c r="B22" t="s">
+        <v>4</v>
+      </c>
+      <c r="C22" t="s">
+        <v>57</v>
+      </c>
+      <c r="D22" t="s">
         <v>58</v>
-      </c>
-      <c r="B22" t="s">
-        <v>4</v>
-      </c>
-      <c r="C22" t="s">
-        <v>59</v>
-      </c>
-      <c r="D22" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B23" t="s">
         <v>4</v>
@@ -916,21 +919,21 @@
         <v>4</v>
       </c>
       <c r="D23" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B24" t="s">
         <v>4</v>
       </c>
       <c r="C24" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="D24" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.2">
@@ -938,13 +941,13 @@
         <v>4</v>
       </c>
       <c r="B25" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C25" t="s">
         <v>4</v>
       </c>
       <c r="D25" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.2">
@@ -952,13 +955,13 @@
         <v>4</v>
       </c>
       <c r="B26" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C26" t="s">
         <v>4</v>
       </c>
       <c r="D26" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.2">
@@ -966,13 +969,13 @@
         <v>4</v>
       </c>
       <c r="B27" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C27" t="s">
         <v>4</v>
       </c>
       <c r="D27" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.2">
@@ -980,13 +983,13 @@
         <v>4</v>
       </c>
       <c r="B28" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C28" t="s">
         <v>4</v>
       </c>
       <c r="D28" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.2">
@@ -994,13 +997,13 @@
         <v>4</v>
       </c>
       <c r="B29" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C29" t="s">
         <v>4</v>
       </c>
       <c r="D29" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
   </sheetData>

</xml_diff>